<commit_message>
Make the two corporation tax rows describe the accounting period
Admin rows 6 and 7 held the accounting period and the year after it, so
the working sheet split the chargeable profit in half and charged half of
it outside the period. Row 6 now runs from the period start to the 31
March inside the period, row 7 from the day after that to the year end,
and a period wholly inside one financial year leaves row 7 empty. K6 and
K7 name the financial year each row belongs to, which is the calendar
year its 1 April fell in.

The six formula cells carry cached values a spreadsheet app reads when it
updates links against a closed Financialaccounts.xlsx, so the generator
rolls them to the package's own year end. Fixedassets caches the same
Admin cells on its side of the link and carried the template's snapshot
for every package; it now gets rolled too.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/templates/ltd/Financialaccounts.xlsx
+++ b/app/templates/ltd/Financialaccounts.xlsx
@@ -16422,7 +16422,7 @@
       </c>
       <c r="J6" s="185"/>
       <c r="K6" s="185">
-        <f>YEAR(L6)</f>
+        <f>YEAR(L6)-IF(MONTH(L6)&lt;4,1,0)</f>
         <v>2025</v>
       </c>
       <c r="L6" s="638">
@@ -16431,7 +16431,7 @@
       </c>
       <c r="M6" s="639"/>
       <c r="N6" s="638">
-        <f>B32</f>
+        <f>MIN(IF(DATE(YEAR(L6),3,31)&gt;=L6,DATE(YEAR(L6),3,31),DATE(YEAR(L6)+1,3,31)),F21)</f>
         <v>46112</v>
       </c>
       <c r="O6" s="641"/>
@@ -16466,17 +16466,17 @@
       </c>
       <c r="J7" s="185"/>
       <c r="K7" s="185">
-        <f>YEAR(L7)</f>
+        <f>YEAR(L7)-IF(MONTH(L7)&lt;4,1,0)</f>
         <v>2026</v>
       </c>
       <c r="L7" s="638">
-        <f>B33</f>
+        <f>N6+1</f>
         <v>46113</v>
       </c>
       <c r="M7" s="639"/>
       <c r="N7" s="638">
-        <f>B56</f>
-        <v>46477</v>
+        <f>F21</f>
+        <v>46112</v>
       </c>
       <c r="O7" s="641"/>
       <c r="P7" s="310">
@@ -44974,8 +44974,8 @@
     </row>
     <row r="34" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A34" s="184">
-        <f>D34-C34+1</f>
-        <v>365</v>
+        <f>MAX(0,D34-C34+1)</f>
+        <v>0</v>
       </c>
       <c r="B34" s="182" t="s">
         <v>14</v>
@@ -45012,7 +45012,7 @@
     <row r="35" spans="1:12" s="40" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A35" s="184">
         <f>D34-C33+1</f>
-        <v>730</v>
+        <v>365</v>
       </c>
       <c r="B35" s="157"/>
       <c r="C35" s="420" t="s">

</xml_diff>

<commit_message>
Wire the CT600's second financial year row and its relief boxes
Boxes 53 to 56 carried no formula, so box 63 filed the first tax row on
its own. They now read the second tax row and blank themselves when the
accounting period lies inside one financial year. Boxes 46 and 56 carry
the tax at the rate before relief, box 64 the relief the working sheet
took off and box 65 the charge the accounts hold, which is also what box
70 self-assesses and what box 66's underlying rate is worked from.

The value field on boxes 64 and 65 is the merged Y to AC block, not the
narrow X pad the plan named. The template's own layout on the unwired
input boxes above them settles it.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/templates/ltd/Financialaccounts.xlsx
+++ b/app/templates/ltd/Financialaccounts.xlsx
@@ -52816,7 +52816,7 @@
         <v>150</v>
       </c>
       <c r="AJ126" s="535">
-        <f>CorporationTax!I33</f>
+        <f>CorporationTax!J33</f>
         <v>0</v>
       </c>
       <c r="AK126" s="535"/>
@@ -52881,12 +52881,15 @@
       <c r="B128" s="209">
         <v>53</v>
       </c>
-      <c r="C128" s="483"/>
-      <c r="D128" s="483"/>
-      <c r="E128" s="483"/>
-      <c r="F128" s="483"/>
-      <c r="G128" s="483"/>
-      <c r="H128" s="483"/>
+      <c r="C128" s="545" t="str">
+        <f>IF(CorporationTax!A34&gt;0,CorporationTax!E34," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="D128" s="546"/>
+      <c r="E128" s="546"/>
+      <c r="F128" s="546"/>
+      <c r="G128" s="546"/>
+      <c r="H128" s="547"/>
       <c r="I128" s="198"/>
       <c r="J128" s="198"/>
       <c r="K128" s="198"/>
@@ -52896,13 +52899,16 @@
       <c r="M128" s="210" t="s">
         <v>150</v>
       </c>
-      <c r="N128" s="483"/>
-      <c r="O128" s="483"/>
-      <c r="P128" s="483"/>
-      <c r="Q128" s="483"/>
-      <c r="R128" s="483"/>
-      <c r="S128" s="483"/>
-      <c r="T128" s="483"/>
+      <c r="N128" s="522" t="str">
+        <f>IF(CorporationTax!A34&gt;0,CorporationTax!F34," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="O128" s="468"/>
+      <c r="P128" s="468"/>
+      <c r="Q128" s="468"/>
+      <c r="R128" s="468"/>
+      <c r="S128" s="468"/>
+      <c r="T128" s="534"/>
       <c r="U128" s="198"/>
       <c r="V128" s="198"/>
       <c r="W128" s="198"/>
@@ -52911,8 +52917,11 @@
         <v>55</v>
       </c>
       <c r="Z128" s="351"/>
-      <c r="AA128" s="483"/>
-      <c r="AB128" s="483"/>
+      <c r="AA128" s="548" t="str">
+        <f>IF(CorporationTax!A34&gt;0,CorporationTax!G34," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="AB128" s="549"/>
       <c r="AC128" s="198"/>
       <c r="AD128" s="198"/>
       <c r="AE128" s="198"/>
@@ -52924,13 +52933,16 @@
       <c r="AI128" s="212" t="s">
         <v>150</v>
       </c>
-      <c r="AJ128" s="535"/>
-      <c r="AK128" s="468"/>
-      <c r="AL128" s="468"/>
-      <c r="AM128" s="468"/>
-      <c r="AN128" s="468"/>
-      <c r="AO128" s="468"/>
-      <c r="AP128" s="468"/>
+      <c r="AJ128" s="535">
+        <f>CorporationTax!J34</f>
+        <v>0</v>
+      </c>
+      <c r="AK128" s="535"/>
+      <c r="AL128" s="535"/>
+      <c r="AM128" s="535"/>
+      <c r="AN128" s="535"/>
+      <c r="AO128" s="535"/>
+      <c r="AP128" s="535"/>
       <c r="AQ128" s="224" t="s">
         <v>391</v>
       </c>
@@ -53168,11 +53180,14 @@
         <v>150</v>
       </c>
       <c r="X133" s="225"/>
-      <c r="Y133" s="514"/>
-      <c r="Z133" s="514"/>
-      <c r="AA133" s="514"/>
-      <c r="AB133" s="514"/>
-      <c r="AC133" s="514"/>
+      <c r="Y133" s="535">
+        <f>CorporationTax!L33+CorporationTax!L34</f>
+        <v>0</v>
+      </c>
+      <c r="Z133" s="535"/>
+      <c r="AA133" s="535"/>
+      <c r="AB133" s="535"/>
+      <c r="AC133" s="535"/>
       <c r="AD133" s="225"/>
       <c r="AE133" s="224" t="s">
         <v>391</v>
@@ -53270,11 +53285,14 @@
         <v>150</v>
       </c>
       <c r="X135" s="225"/>
-      <c r="Y135" s="514"/>
-      <c r="Z135" s="514"/>
-      <c r="AA135" s="514"/>
-      <c r="AB135" s="514"/>
-      <c r="AC135" s="514"/>
+      <c r="Y135" s="535">
+        <f>AJ131-Y133</f>
+        <v>0</v>
+      </c>
+      <c r="Z135" s="535"/>
+      <c r="AA135" s="535"/>
+      <c r="AB135" s="535"/>
+      <c r="AC135" s="535"/>
       <c r="AD135" s="225"/>
       <c r="AE135" s="224" t="s">
         <v>391</v>
@@ -53369,7 +53387,7 @@
         <v>66</v>
       </c>
       <c r="W137" s="543" t="str">
-        <f>IF(AJ131&gt;0,AJ131*100/AJ110," ")</f>
+        <f>IF(Y135&gt;0,Y135*100/AJ110," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="X137" s="544"/>
@@ -53791,7 +53809,7 @@
         <v>150</v>
       </c>
       <c r="AJ145" s="535">
-        <f>AJ131</f>
+        <f>Y135</f>
         <v>0</v>
       </c>
       <c r="AK145" s="468"/>

</xml_diff>

<commit_message>
F9: remove the obsolete expensive-car WDA cap from all four products
The pre-2009 expensive-car restriction (cost threshold + flat WDA cap)
no longer applies. Drop it from the Ltd, SE, BST and Taxi capital
allowance templates, tax-year data, generator writes and compliance
checks, so a motor vehicle claims WDA at the plain main-pool rate with
no cap. Ltd's Schedule rate cell R4 now reads Admin's own WDA rate
(previously a literal 20) so it moves with the tax-year data.
</commit_message>
<xml_diff>
--- a/app/templates/ltd/Financialaccounts.xlsx
+++ b/app/templates/ltd/Financialaccounts.xlsx
@@ -16594,18 +16594,10 @@
         <v>45778</v>
       </c>
       <c r="C11" s="253"/>
-      <c r="D11" s="253" t="s">
-        <v>501</v>
-      </c>
-      <c r="E11" s="262">
-        <v>12000</v>
-      </c>
-      <c r="F11" s="253" t="s">
-        <v>502</v>
-      </c>
-      <c r="G11" s="262">
-        <v>3000</v>
-      </c>
+      <c r="D11" s="253"/>
+      <c r="E11" s="262"/>
+      <c r="F11" s="253"/>
+      <c r="G11" s="262"/>
       <c r="H11" s="253"/>
       <c r="I11" s="253"/>
       <c r="J11" s="253"/>

</xml_diff>

<commit_message>
Fix Ltd CT600 capital-allowance schedule to read CorporationTax column I
AA177, AL177 and AA179 (the CT600 sheet's boxes 107/108 and 109, general
pool allowances/balancing charge and cars outside the pool) referenced
CorporationTax!H15-H18, a column the working sheet never populates,
so these three cells printed blank on every package. The allowances sit
in column I. Repointed all three formulas at column I; nothing else in
the sheet or workbook changed.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ctg3ZH834LyPxhnJcLYgcJ
</commit_message>
<xml_diff>
--- a/app/templates/ltd/Financialaccounts.xlsx
+++ b/app/templates/ltd/Financialaccounts.xlsx
@@ -55397,7 +55397,7 @@
         <v>150</v>
       </c>
       <c r="AA177" s="522" t="str">
-        <f>IF((CorporationTax!H15+CorporationTax!H17)&gt;0,CorporationTax!H15+CorporationTax!H17," ")</f>
+        <f>IF((CorporationTax!I15+CorporationTax!I17)&gt;0,CorporationTax!I15+CorporationTax!I17," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="AB177" s="522"/>
@@ -55415,7 +55415,7 @@
         <v>150</v>
       </c>
       <c r="AL177" s="522" t="str">
-        <f>IF(CorporationTax!H18&lt;&gt;0,CorporationTax!H18," ")</f>
+        <f>IF(CorporationTax!I18&lt;&gt;0,CorporationTax!I18," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="AM177" s="522"/>
@@ -55507,7 +55507,7 @@
         <v>150</v>
       </c>
       <c r="AA179" s="522" t="str">
-        <f>IF(CorporationTax!H16&gt;0,CorporationTax!H16," ")</f>
+        <f>IF(CorporationTax!I16&gt;0,CorporationTax!I16," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="AB179" s="522"/>

</xml_diff>

<commit_message>
Each product's front sheet states the copyright and the licence
Two shared strings appended and two cells added below the last used row of
Home, Business Details and OpenAccounts: BST and Taxi at B22 and B23, Self
Employed at A58 and A59, the Company hub at B88 and B89. Nothing else in any
package moves. Every other zip part of every generated file is byte for byte
what it was, and the four report.json extractions are identical.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016EA8xMoZDjp49aJHToWYTm
</commit_message>
<xml_diff>
--- a/app/templates/ltd/Financialaccounts.xlsx
+++ b/app/templates/ltd/Financialaccounts.xlsx
@@ -109,7 +109,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1027" uniqueCount="624">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1029" uniqueCount="626">
   <si>
     <t>Depreciation</t>
   </si>
@@ -2159,6 +2159,12 @@
   </si>
   <si>
     <t>(Small profits rate)</t>
+  </si>
+  <si>
+    <t>Copyright (C) 2006-2026 DIY Accounting Limited</t>
+  </si>
+  <si>
+    <t>Licensed under the PolyForm Internal Use License 1.0.0 with an additional grant for accountants. Free to use, source available: https://spreadsheets.diyaccounting.co.uk</t>
   </si>
 </sst>
 </file>
@@ -11957,7 +11963,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:R86"/>
+  <dimension ref="A1:R89"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="11" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="0.83203125" style="6" customWidth="1"/>
@@ -13448,6 +13454,16 @@
       <c r="F86" s="3"/>
       <c r="G86" s="3"/>
       <c r="H86" s="3"/>
+    </row>
+    <row r="88">
+      <c r="B88" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" t="s">
+        <v>625</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="19">

</xml_diff>